<commit_message>
Reference the quencher potentials to SCE at 4.42 V, as the photocatalysts are
quencher_dft.py converted dG_Ox and dG_Red to V vs SCE with an offset of
4.442 V, while photocatalyst_dft.py uses 4.42 V for the excited-state
potentials, so the two sides of every calculated SET driving force sat on
references 0.022 V apart. Both now use 4.42 V.

E_Ox_vs_SCE_calc and E_Red_vs_SCE_calc move up by 0.02 or 0.03 V, the
original's two-decimal rounding kept. dG_SET_calc in exp_dataset changes
in every pair, by up to 0.69 kcal/mol: more endergonic on the oxidation
channel, more exergonic on the reduction channel, less where the more
accessible channel switches. Nothing else in the dataset changes, and no
benchmark result changes: the default run makes no mechanism decision and
never reads dG_SET.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/quencher_properties_calc.xlsx
+++ b/data/computational_data_processed/quencher_properties_calc.xlsx
@@ -795,7 +795,7 @@
         <v>144.5</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>1.82</v>
+        <v>1.85</v>
       </c>
       <c r="L3" s="19" t="n">
         <v>4.5</v>
@@ -807,7 +807,7 @@
         <v>49.9</v>
       </c>
       <c r="P3" s="19" t="n">
-        <v>-2.28</v>
+        <v>-2.26</v>
       </c>
       <c r="Q3" s="19" t="n">
         <v>4.9</v>
@@ -896,7 +896,7 @@
         <v>142.9</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>1.75</v>
+        <v>1.78</v>
       </c>
       <c r="L4" s="19" t="n">
         <v>4.4</v>
@@ -908,7 +908,7 @@
         <v>41.4</v>
       </c>
       <c r="P4" s="19" t="n">
-        <v>-2.65</v>
+        <v>-2.62</v>
       </c>
       <c r="Q4" s="19" t="n">
         <v>5.5</v>
@@ -997,7 +997,7 @@
         <v>155.5</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>2.3</v>
+        <v>2.32</v>
       </c>
       <c r="L5" s="19" t="n">
         <v>5.3</v>
@@ -1009,7 +1009,7 @@
         <v>73</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>-1.28</v>
+        <v>-1.25</v>
       </c>
       <c r="Q5" s="19" t="n">
         <v>12.9</v>
@@ -1098,7 +1098,7 @@
         <v>139.5</v>
       </c>
       <c r="K6" s="19" t="n">
-        <v>1.61</v>
+        <v>1.63</v>
       </c>
       <c r="L6" s="19" t="n">
         <v>3.9</v>
@@ -1110,7 +1110,7 @@
         <v>35.4</v>
       </c>
       <c r="P6" s="19" t="n">
-        <v>-2.91</v>
+        <v>-2.88</v>
       </c>
       <c r="Q6" s="19" t="n">
         <v>5.1</v>
@@ -1199,7 +1199,7 @@
         <v>158.8</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>2.44</v>
+        <v>2.47</v>
       </c>
       <c r="L7" s="19" t="n">
         <v>10.1</v>
@@ -1211,7 +1211,7 @@
         <v>63.9</v>
       </c>
       <c r="P7" s="19" t="n">
-        <v>-1.67</v>
+        <v>-1.65</v>
       </c>
       <c r="Q7" s="19" t="n">
         <v>4.8</v>
@@ -1300,7 +1300,7 @@
         <v>145.5</v>
       </c>
       <c r="K8" s="19" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="L8" s="19" t="n">
         <v>3.4</v>
@@ -1312,7 +1312,7 @@
         <v>49.6</v>
       </c>
       <c r="P8" s="19" t="n">
-        <v>-2.29</v>
+        <v>-2.27</v>
       </c>
       <c r="Q8" s="19" t="n">
         <v>4.7</v>
@@ -1401,7 +1401,7 @@
         <v>151.3</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="L9" s="19" t="n">
         <v>3.8</v>
@@ -1413,7 +1413,7 @@
         <v>60.3</v>
       </c>
       <c r="P9" s="19" t="n">
-        <v>-1.83</v>
+        <v>-1.81</v>
       </c>
       <c r="Q9" s="19" t="n">
         <v>6.7</v>
@@ -1502,7 +1502,7 @@
         <v>158.2</v>
       </c>
       <c r="K10" s="19" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="L10" s="19" t="n">
         <v>24.4</v>
@@ -1514,7 +1514,7 @@
         <v>54.8</v>
       </c>
       <c r="P10" s="19" t="n">
-        <v>-2.07</v>
+        <v>-2.04</v>
       </c>
       <c r="Q10" s="19" t="n">
         <v>11.3</v>
@@ -1603,7 +1603,7 @@
         <v>134.8</v>
       </c>
       <c r="K11" s="19" t="n">
-        <v>1.4</v>
+        <v>1.43</v>
       </c>
       <c r="L11" s="19" t="n">
         <v>6</v>
@@ -1615,7 +1615,7 @@
         <v>39.1</v>
       </c>
       <c r="P11" s="19" t="n">
-        <v>-2.75</v>
+        <v>-2.72</v>
       </c>
       <c r="Q11" s="19" t="n">
         <v>7.4</v>
@@ -1704,7 +1704,7 @@
         <v>137.6</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="L12" s="19" t="n">
         <v>10.5</v>
@@ -1797,7 +1797,7 @@
         <v>136.7</v>
       </c>
       <c r="K13" s="19" t="n">
-        <v>1.49</v>
+        <v>1.51</v>
       </c>
       <c r="L13" s="19" t="n">
         <v>9.300000000000001</v>
@@ -1890,7 +1890,7 @@
         <v>140.9</v>
       </c>
       <c r="K14" s="19" t="n">
-        <v>1.67</v>
+        <v>1.69</v>
       </c>
       <c r="L14" s="19" t="n">
         <v>4.6</v>
@@ -1902,7 +1902,7 @@
         <v>44.5</v>
       </c>
       <c r="P14" s="19" t="n">
-        <v>-2.51</v>
+        <v>-2.49</v>
       </c>
       <c r="Q14" s="19" t="n">
         <v>5.1</v>
@@ -1991,7 +1991,7 @@
         <v>172.2</v>
       </c>
       <c r="K15" s="19" t="n">
-        <v>3.03</v>
+        <v>3.05</v>
       </c>
       <c r="L15" s="19" t="n">
         <v>8.9</v>
@@ -2003,7 +2003,7 @@
         <v>76.09999999999999</v>
       </c>
       <c r="P15" s="19" t="n">
-        <v>-1.14</v>
+        <v>-1.12</v>
       </c>
       <c r="Q15" s="19" t="n">
         <v>9.300000000000001</v>
@@ -2092,7 +2092,7 @@
         <v>159</v>
       </c>
       <c r="K16" s="19" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="L16" s="19" t="n">
         <v>90.90000000000001</v>
@@ -2104,7 +2104,7 @@
         <v>48</v>
       </c>
       <c r="P16" s="19" t="n">
-        <v>-2.36</v>
+        <v>-2.34</v>
       </c>
       <c r="Q16" s="19" t="n">
         <v>11</v>
@@ -2193,7 +2193,7 @@
         <v>136.3</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
       <c r="L17" s="19" t="n">
         <v>4.3</v>
@@ -2205,7 +2205,7 @@
         <v>32.7</v>
       </c>
       <c r="P17" s="19" t="n">
-        <v>-3.02</v>
+        <v>-3</v>
       </c>
       <c r="Q17" s="19" t="n">
         <v>5.9</v>
@@ -2294,7 +2294,7 @@
         <v>134.5</v>
       </c>
       <c r="K18" s="19" t="n">
-        <v>1.39</v>
+        <v>1.41</v>
       </c>
       <c r="L18" s="19" t="n">
         <v>5.5</v>
@@ -2306,7 +2306,7 @@
         <v>45.5</v>
       </c>
       <c r="P18" s="19" t="n">
-        <v>-2.47</v>
+        <v>-2.45</v>
       </c>
       <c r="Q18" s="19" t="n">
         <v>6.3</v>
@@ -2395,7 +2395,7 @@
         <v>132.9</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>1.32</v>
+        <v>1.34</v>
       </c>
       <c r="L19" s="19" t="n">
         <v>7.5</v>
@@ -2407,7 +2407,7 @@
         <v>54.2</v>
       </c>
       <c r="P19" s="19" t="n">
-        <v>-2.09</v>
+        <v>-2.07</v>
       </c>
       <c r="Q19" s="19" t="n">
         <v>119.6</v>
@@ -2496,7 +2496,7 @@
         <v>124.5</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="L20" s="19" t="n">
         <v>10.4</v>
@@ -2508,7 +2508,7 @@
         <v>44</v>
       </c>
       <c r="P20" s="19" t="n">
-        <v>-2.53</v>
+        <v>-2.51</v>
       </c>
       <c r="Q20" s="19" t="n">
         <v>7.2</v>
@@ -2597,7 +2597,7 @@
         <v>153</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>2.19</v>
+        <v>2.21</v>
       </c>
       <c r="L21" s="19" t="n">
         <v>5.5</v>
@@ -2609,7 +2609,7 @@
         <v>57.1</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>-1.97</v>
+        <v>-1.94</v>
       </c>
       <c r="Q21" s="19" t="n">
         <v>10.6</v>
@@ -2698,7 +2698,7 @@
         <v>138.8</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="L22" s="19" t="n">
         <v>3</v>
@@ -2710,7 +2710,7 @@
         <v>41.8</v>
       </c>
       <c r="P22" s="19" t="n">
-        <v>-2.63</v>
+        <v>-2.61</v>
       </c>
       <c r="Q22" s="19" t="n">
         <v>4</v>
@@ -2799,7 +2799,7 @@
         <v>155.8</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>2.31</v>
+        <v>2.34</v>
       </c>
       <c r="L23" s="19" t="n">
         <v>5</v>
@@ -2811,7 +2811,7 @@
         <v>56.7</v>
       </c>
       <c r="P23" s="19" t="n">
-        <v>-1.98</v>
+        <v>-1.96</v>
       </c>
       <c r="Q23" s="19" t="n">
         <v>7.3</v>
@@ -2900,7 +2900,7 @@
         <v>148.9</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>2.01</v>
+        <v>2.04</v>
       </c>
       <c r="L24" s="19" t="n">
         <v>6</v>
@@ -2912,7 +2912,7 @@
         <v>57.2</v>
       </c>
       <c r="P24" s="19" t="n">
-        <v>-1.96</v>
+        <v>-1.94</v>
       </c>
       <c r="Q24" s="19" t="n">
         <v>12.2</v>
@@ -3001,7 +3001,7 @@
         <v>140.7</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
       <c r="L25" s="19" t="n">
         <v>3.9</v>
@@ -3013,7 +3013,7 @@
         <v>45.5</v>
       </c>
       <c r="P25" s="19" t="n">
-        <v>-2.47</v>
+        <v>-2.45</v>
       </c>
       <c r="Q25" s="19" t="n">
         <v>6.5</v>
@@ -3102,7 +3102,7 @@
         <v>142.3</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>1.73</v>
+        <v>1.75</v>
       </c>
       <c r="L26" s="19" t="n">
         <v>5.3</v>
@@ -3114,7 +3114,7 @@
         <v>42.7</v>
       </c>
       <c r="P26" s="19" t="n">
-        <v>-2.59</v>
+        <v>-2.57</v>
       </c>
       <c r="Q26" s="19" t="n">
         <v>6.9</v>
@@ -3203,7 +3203,7 @@
         <v>141.3</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
       <c r="L27" s="19" t="n">
         <v>4.6</v>
@@ -3215,7 +3215,7 @@
         <v>64.59999999999999</v>
       </c>
       <c r="P27" s="19" t="n">
-        <v>-1.64</v>
+        <v>-1.62</v>
       </c>
       <c r="Q27" s="19" t="n">
         <v>73.09999999999999</v>
@@ -3304,7 +3304,7 @@
         <v>140.8</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>1.66</v>
+        <v>1.69</v>
       </c>
       <c r="L28" s="19" t="n">
         <v>5.1</v>
@@ -3316,7 +3316,7 @@
         <v>62.2</v>
       </c>
       <c r="P28" s="19" t="n">
-        <v>-1.74</v>
+        <v>-1.72</v>
       </c>
       <c r="Q28" s="19" t="n">
         <v>73.5</v>
@@ -3405,7 +3405,7 @@
         <v>144.2</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="L29" s="19" t="n">
         <v>5.3</v>
@@ -3417,7 +3417,7 @@
         <v>65.3</v>
       </c>
       <c r="P29" s="19" t="n">
-        <v>-1.61</v>
+        <v>-1.59</v>
       </c>
       <c r="Q29" s="19" t="n">
         <v>68</v>
@@ -3506,7 +3506,7 @@
         <v>159.3</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>2.47</v>
+        <v>2.49</v>
       </c>
       <c r="L30" s="19" t="n">
         <v>6.3</v>
@@ -3518,7 +3518,7 @@
         <v>71</v>
       </c>
       <c r="P30" s="19" t="n">
-        <v>-1.36</v>
+        <v>-1.34</v>
       </c>
       <c r="Q30" s="19" t="n">
         <v>6.6</v>
@@ -3607,7 +3607,7 @@
         <v>154.9</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>2.27</v>
+        <v>2.3</v>
       </c>
       <c r="L31" s="19" t="n">
         <v>7.9</v>
@@ -3619,7 +3619,7 @@
         <v>55</v>
       </c>
       <c r="P31" s="19" t="n">
-        <v>-2.06</v>
+        <v>-2.04</v>
       </c>
       <c r="Q31" s="19" t="n">
         <v>7</v>
@@ -3708,7 +3708,7 @@
         <v>132.6</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>1.31</v>
+        <v>1.33</v>
       </c>
       <c r="L32" s="19" t="n">
         <v>4.8</v>
@@ -3720,7 +3720,7 @@
         <v>49.3</v>
       </c>
       <c r="P32" s="19" t="n">
-        <v>-2.3</v>
+        <v>-2.28</v>
       </c>
       <c r="Q32" s="19" t="n">
         <v>5.4</v>
@@ -3809,7 +3809,7 @@
         <v>142.4</v>
       </c>
       <c r="K33" s="19" t="n">
-        <v>1.73</v>
+        <v>1.75</v>
       </c>
       <c r="L33" s="19" t="n">
         <v>7.4</v>
@@ -3821,7 +3821,7 @@
         <v>40.2</v>
       </c>
       <c r="P33" s="19" t="n">
-        <v>-2.7</v>
+        <v>-2.68</v>
       </c>
       <c r="Q33" s="19" t="n">
         <v>27.2</v>
@@ -3910,7 +3910,7 @@
         <v>134.1</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>1.37</v>
+        <v>1.4</v>
       </c>
       <c r="L34" s="19" t="n">
         <v>2.5</v>
@@ -3922,7 +3922,7 @@
         <v>53.8</v>
       </c>
       <c r="P34" s="19" t="n">
-        <v>-2.11</v>
+        <v>-2.09</v>
       </c>
       <c r="Q34" s="19" t="n">
         <v>21.1</v>
@@ -4011,7 +4011,7 @@
         <v>133.5</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="L35" s="19" t="n">
         <v>7.2</v>
@@ -4023,7 +4023,7 @@
         <v>51.3</v>
       </c>
       <c r="P35" s="19" t="n">
-        <v>-2.22</v>
+        <v>-2.2</v>
       </c>
       <c r="Q35" s="19" t="n">
         <v>23.5</v>
@@ -4112,7 +4112,7 @@
         <v>139.8</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>1.62</v>
+        <v>1.64</v>
       </c>
       <c r="L36" s="19" t="n">
         <v>13.6</v>
@@ -4124,7 +4124,7 @@
         <v>44</v>
       </c>
       <c r="P36" s="19" t="n">
-        <v>-2.53</v>
+        <v>-2.51</v>
       </c>
       <c r="Q36" s="19" t="n">
         <v>8.199999999999999</v>
@@ -4213,7 +4213,7 @@
         <v>135.6</v>
       </c>
       <c r="K37" s="19" t="n">
-        <v>1.44</v>
+        <v>1.46</v>
       </c>
       <c r="L37" s="19" t="n">
         <v>8.6</v>
@@ -4225,7 +4225,7 @@
         <v>52.8</v>
       </c>
       <c r="P37" s="19" t="n">
-        <v>-2.15</v>
+        <v>-2.13</v>
       </c>
       <c r="Q37" s="19" t="n">
         <v>1.9</v>
@@ -4314,7 +4314,7 @@
         <v>138.4</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>1.56</v>
+        <v>1.58</v>
       </c>
       <c r="L38" s="19" t="n">
         <v>4.6</v>
@@ -4326,7 +4326,7 @@
         <v>44.9</v>
       </c>
       <c r="P38" s="19" t="n">
-        <v>-2.49</v>
+        <v>-2.47</v>
       </c>
       <c r="Q38" s="19" t="n">
         <v>6.9</v>
@@ -4415,7 +4415,7 @@
         <v>143.1</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>1.76</v>
+        <v>1.79</v>
       </c>
       <c r="L39" s="19" t="n">
         <v>6</v>
@@ -4427,7 +4427,7 @@
         <v>44.7</v>
       </c>
       <c r="P39" s="19" t="n">
-        <v>-2.5</v>
+        <v>-2.48</v>
       </c>
       <c r="Q39" s="19" t="n">
         <v>26.9</v>
@@ -4516,7 +4516,7 @@
         <v>145.6</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="L40" s="19" t="n">
         <v>4.5</v>
@@ -4528,7 +4528,7 @@
         <v>41.6</v>
       </c>
       <c r="P40" s="19" t="n">
-        <v>-2.64</v>
+        <v>-2.62</v>
       </c>
       <c r="Q40" s="19" t="n">
         <v>8.9</v>
@@ -4617,7 +4617,7 @@
         <v>139</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>1.59</v>
+        <v>1.61</v>
       </c>
       <c r="L41" s="19" t="n">
         <v>7</v>
@@ -4629,7 +4629,7 @@
         <v>49.9</v>
       </c>
       <c r="P41" s="19" t="n">
-        <v>-2.28</v>
+        <v>-2.26</v>
       </c>
       <c r="Q41" s="19" t="n">
         <v>5.5</v>
@@ -4718,7 +4718,7 @@
         <v>144</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>1.8</v>
+        <v>1.82</v>
       </c>
       <c r="L42" s="19" t="n">
         <v>6.5</v>
@@ -4730,7 +4730,7 @@
         <v>45.7</v>
       </c>
       <c r="P42" s="19" t="n">
-        <v>-2.46</v>
+        <v>-2.44</v>
       </c>
       <c r="Q42" s="19" t="n">
         <v>5.8</v>
@@ -4819,7 +4819,7 @@
         <v>141.3</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
       <c r="L43" s="19" t="n">
         <v>5.1</v>
@@ -4831,7 +4831,7 @@
         <v>39.5</v>
       </c>
       <c r="P43" s="19" t="n">
-        <v>-2.73</v>
+        <v>-2.71</v>
       </c>
       <c r="Q43" s="19" t="n">
         <v>6.1</v>
@@ -4920,7 +4920,7 @@
         <v>150.9</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>2.1</v>
+        <v>2.12</v>
       </c>
       <c r="L44" s="19" t="n">
         <v>7.1</v>
@@ -4932,7 +4932,7 @@
         <v>61.4</v>
       </c>
       <c r="P44" s="19" t="n">
-        <v>-1.78</v>
+        <v>-1.76</v>
       </c>
       <c r="Q44" s="19" t="n">
         <v>7</v>
@@ -5021,7 +5021,7 @@
         <v>147.3</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="L45" s="19" t="n">
         <v>6</v>
@@ -5033,7 +5033,7 @@
         <v>57.1</v>
       </c>
       <c r="P45" s="19" t="n">
-        <v>-1.97</v>
+        <v>-1.94</v>
       </c>
       <c r="Q45" s="19" t="n">
         <v>6.9</v>
@@ -5122,7 +5122,7 @@
         <v>161.4</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>2.56</v>
+        <v>2.58</v>
       </c>
       <c r="L46" s="19" t="n">
         <v>11.4</v>
@@ -5134,7 +5134,7 @@
         <v>60.1</v>
       </c>
       <c r="P46" s="19" t="n">
-        <v>-1.84</v>
+        <v>-1.81</v>
       </c>
       <c r="Q46" s="19" t="n">
         <v>7.8</v>
@@ -5223,7 +5223,7 @@
         <v>152.6</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="L47" s="19" t="n">
         <v>6</v>
@@ -5235,7 +5235,7 @@
         <v>46.4</v>
       </c>
       <c r="P47" s="19" t="n">
-        <v>-2.43</v>
+        <v>-2.41</v>
       </c>
       <c r="Q47" s="19" t="n">
         <v>12.2</v>
@@ -5324,7 +5324,7 @@
         <v>145.4</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>1.86</v>
+        <v>1.89</v>
       </c>
       <c r="L48" s="19" t="n">
         <v>31.1</v>
@@ -5336,7 +5336,7 @@
         <v>51.7</v>
       </c>
       <c r="P48" s="19" t="n">
-        <v>-2.2</v>
+        <v>-2.18</v>
       </c>
       <c r="Q48" s="19" t="n">
         <v>6.1</v>
@@ -5425,7 +5425,7 @@
         <v>152.7</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="L49" s="19" t="n">
         <v>25.6</v>
@@ -5437,7 +5437,7 @@
         <v>58.2</v>
       </c>
       <c r="P49" s="19" t="n">
-        <v>-1.92</v>
+        <v>-1.9</v>
       </c>
       <c r="Q49" s="19" t="n">
         <v>7.8</v>
@@ -5526,7 +5526,7 @@
         <v>158.9</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="L50" s="19" t="n">
         <v>4</v>
@@ -5538,7 +5538,7 @@
         <v>51.9</v>
       </c>
       <c r="P50" s="19" t="n">
-        <v>-2.19</v>
+        <v>-2.17</v>
       </c>
       <c r="Q50" s="19" t="n">
         <v>8.699999999999999</v>
@@ -5869,7 +5869,7 @@
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>dG_Ox / F - 4.442 V.</t>
+          <t>dG_Ox / F - 4.42 V.</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>dG_Red / F - 4.442 V.</t>
+          <t>dG_Red / F - 4.42 V.</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Name the quenchers from their SMILES
The quencher names came from the lab record: shorthand such as
"OiPr bifunc" and "Br-Benzothiophen", German spellings, and in one case a
different compound ("maleimide" for N-methylmaleimide). They are now
derived from the SMILES, in QUENCHER_NAME in compound_records.py, and each
was checked by converting it back to a structure with OPSIN: all 48
match their SMILES, stereo included. The lab label is kept as lab_label
in the raw intermediate.

The Stern-Volmer pipetting maps label seven quenchers as thiazoles or
oxazoles that the records, the SMILES and the recorded molar masses show
are thiophenes and furans (Q9, Q23-26, Q42, Q43). Their labels are no
longer carried into stern_volmer_intensities.csv, and the absorption table
drops its own name column; quencher ids carry identity there, and names
live in the records and the workbooks.

Both quencher workbooks and the ML prediction table carry the new names.
No measured or computed value changes.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/quencher_properties_calc.xlsx
+++ b/data/computational_data_processed/quencher_properties_calc.xlsx
@@ -513,7 +513,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="2" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>6-Me-quinoline</t>
+          <t>6-methylquinoline</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>2-Nitro-m-Xylene</t>
+          <t>1,3-dimethyl-2-nitrobenzene</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Benzothiophene</t>
+          <t>benzo[b]thiophene</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Quinoxaline</t>
+          <t>quinoxaline</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Isoquinoline</t>
+          <t>isoquinoline</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Coumarin</t>
+          <t>coumarin</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>OiPr bifunc</t>
+          <t>benzophenone O-(isopropoxycarbonyl) oxime</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>2-Ph-3-Me-Thiazol</t>
+          <t>3-methyl-2-phenylthiophene</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Diphenyldisulfide</t>
+          <t>diphenyl disulfide</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Dibenzyldisulfide</t>
+          <t>dibenzyl disulfide</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>dihydro azaborinine</t>
+          <t>1,2-dihydro-1,2-benzazaborinine</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>maleimide</t>
+          <t>N-methylmaleimide</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Butyl-Methacrylate</t>
+          <t>butyl methacrylate</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Inden</t>
+          <t>indene</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>5-Me-Pyridone</t>
+          <t>5-methylpyridin-2(1H)-one</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>(BnSe)2</t>
+          <t>dibenzyl diselenide</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>oxadiazole</t>
+          <t>5,5-dimethyl-3-phenyl-4,5-dihydro-1,2,4-oxadiazole</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>sulfur bifunc</t>
+          <t>benzophenone O-[(benzylsulfanyl)carbonyl] oxime</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Ethylphenylpropiolat</t>
+          <t>ethyl 3-phenylpropiolate</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>4-Oxo-Quinazolin</t>
+          <t>4-oxo-2-phenylquinazolin-3(4H)-yl 3-phenylpropanoate</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Bpin-Benzothiophen</t>
+          <t>2-(benzo[b]thiophen-2-yl)-4,4,5,5-tetramethyl-1,3,2-dioxaborolane</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>Bpin-Benzofuran</t>
+          <t>2-(benzofuran-2-yl)-4,4,5,5-tetramethyl-1,3,2-dioxaborolane</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Br-Benzothiophen</t>
+          <t>2-bromobenzo[b]thiophene</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>Br-Benzofuran</t>
+          <t>2-bromobenzofuran</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Di-Br-Thiophene</t>
+          <t>2,5-dibromothiophene</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Benzoyl-Thiazol</t>
+          <t>2-benzoylthiazole</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Isoxazolon</t>
+          <t>4,4-dimethyl-3-phenylisoxazol-5(4H)-one</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>E-Stilbene</t>
+          <t>(E)-stilbene</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>N-Peroxide</t>
+          <t>6-phenyl-5-oxa-6-azaspiro[2.4]heptane-4,7-dione</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Thioamide 1</t>
+          <t>1-(thiobenzoyl)pyrrolidine</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Thioamide 2</t>
+          <t>N-methyl-N-phenylpropanethioamide</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>oxime ether</t>
+          <t>(Z)-3,4-dihydronaphthalen-1(2H)-one O-methyl oxime</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Z-Stilbene</t>
+          <t>(Z)-stilbene</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Ac-Pyrol</t>
+          <t>2-acetyl-1-methylpyrrole</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>F-styrene</t>
+          <t>1-bromo-4-(2,2-difluorovinyl)benzene</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>butadiene</t>
+          <t>1,3-butadiene</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>4-Me-2-Ph-Thiazol</t>
+          <t>4-methyl-2-phenylthiazole</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Ph-Oxazol</t>
+          <t>2-phenyloxazole</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>alpha-Methylstyrol</t>
+          <t>alpha-methylstyrene</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>2-Benzoyl-Furan</t>
+          <t>2-benzoylfuran</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>2-Acetyl-4-Me-Thiophen</t>
+          <t>2-acetyl-4-methylthiophene</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>2-Acetylpyridine</t>
+          <t>2-acetylpyridine</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>vinyl selenoxide</t>
+          <t>phenyl vinyl selenoxide</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Azirin-Intermediat</t>
+          <t>2,2-dimethyl-3-phenyl-2H-azirine</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Quinolin-8-Ester</t>
+          <t>methyl quinoline-8-carboxylate</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Cyclohexenone</t>
+          <t>cyclohex-2-en-1-one</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -5711,7 +5711,7 @@
       <c r="C4" s="21" t="inlineStr"/>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>Compound, from the experimental record.</t>
+          <t>Name derived from the SMILES, as in the experimental workbook.</t>
         </is>
       </c>
       <c r="E4" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Store the quencher reduction free energy as G(Q-) - G(Q)
dG_Red now has the sign of the photocatalyst table and of SI section 3.1. The reduction
potentials are unchanged.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/quencher_properties_calc.xlsx
+++ b/data/computational_data_processed/quencher_properties_calc.xlsx
@@ -782,7 +782,7 @@
         <v>4.14</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>49.93</v>
+        <v>-49.93</v>
       </c>
       <c r="P3" s="18" t="n">
         <v>-2.25</v>
@@ -874,7 +874,7 @@
         <v>4.39</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>41.41</v>
+        <v>-41.41</v>
       </c>
       <c r="P4" s="18" t="n">
         <v>-2.62</v>
@@ -966,7 +966,7 @@
         <v>11</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>73.03</v>
+        <v>-73.03</v>
       </c>
       <c r="P5" s="18" t="n">
         <v>-1.25</v>
@@ -1058,7 +1058,7 @@
         <v>3.58</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>35.44</v>
+        <v>-35.44</v>
       </c>
       <c r="P6" s="18" t="n">
         <v>-2.88</v>
@@ -1150,7 +1150,7 @@
         <v>3.49</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>63.87</v>
+        <v>-63.87</v>
       </c>
       <c r="P7" s="18" t="n">
         <v>-1.65</v>
@@ -1242,7 +1242,7 @@
         <v>3.5</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>49.56</v>
+        <v>-49.56</v>
       </c>
       <c r="P8" s="18" t="n">
         <v>-2.27</v>
@@ -1334,7 +1334,7 @@
         <v>3.83</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>60.27</v>
+        <v>-60.27</v>
       </c>
       <c r="P9" s="18" t="n">
         <v>-1.81</v>
@@ -1426,7 +1426,7 @@
         <v>5.93</v>
       </c>
       <c r="O10" s="18" t="n">
-        <v>54.84</v>
+        <v>-54.84</v>
       </c>
       <c r="P10" s="18" t="n">
         <v>-2.04</v>
@@ -1518,7 +1518,7 @@
         <v>6.87</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>39.09</v>
+        <v>-39.09</v>
       </c>
       <c r="P11" s="18" t="n">
         <v>-2.73</v>
@@ -1778,7 +1778,7 @@
         <v>4.57</v>
       </c>
       <c r="O14" s="18" t="n">
-        <v>44.5</v>
+        <v>-44.5</v>
       </c>
       <c r="P14" s="18" t="n">
         <v>-2.49</v>
@@ -1870,7 +1870,7 @@
         <v>6.92</v>
       </c>
       <c r="O15" s="18" t="n">
-        <v>76.12</v>
+        <v>-76.12</v>
       </c>
       <c r="P15" s="18" t="n">
         <v>-1.12</v>
@@ -1962,7 +1962,7 @@
         <v>7.49</v>
       </c>
       <c r="O16" s="18" t="n">
-        <v>48</v>
+        <v>-48</v>
       </c>
       <c r="P16" s="18" t="n">
         <v>-2.34</v>
@@ -2054,7 +2054,7 @@
         <v>4.37</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>32.73</v>
+        <v>-32.73</v>
       </c>
       <c r="P17" s="18" t="n">
         <v>-3</v>
@@ -2146,7 +2146,7 @@
         <v>4.35</v>
       </c>
       <c r="O18" s="18" t="n">
-        <v>45.51</v>
+        <v>-45.51</v>
       </c>
       <c r="P18" s="18" t="n">
         <v>-2.45</v>
@@ -2238,7 +2238,7 @@
         <v>13.69</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>54.16</v>
+        <v>-54.16</v>
       </c>
       <c r="P19" s="18" t="n">
         <v>-2.07</v>
@@ -2330,7 +2330,7 @@
         <v>13.82</v>
       </c>
       <c r="O20" s="18" t="n">
-        <v>43.96</v>
+        <v>-43.96</v>
       </c>
       <c r="P20" s="18" t="n">
         <v>-2.51</v>
@@ -2422,7 +2422,7 @@
         <v>4.64</v>
       </c>
       <c r="O21" s="18" t="n">
-        <v>57.15</v>
+        <v>-57.15</v>
       </c>
       <c r="P21" s="18" t="n">
         <v>-1.94</v>
@@ -2514,7 +2514,7 @@
         <v>3.03</v>
       </c>
       <c r="O22" s="18" t="n">
-        <v>41.8</v>
+        <v>-41.8</v>
       </c>
       <c r="P22" s="18" t="n">
         <v>-2.61</v>
@@ -2606,7 +2606,7 @@
         <v>5.32</v>
       </c>
       <c r="O23" s="18" t="n">
-        <v>56.74</v>
+        <v>-56.74</v>
       </c>
       <c r="P23" s="18" t="n">
         <v>-1.96</v>
@@ -2698,7 +2698,7 @@
         <v>7.13</v>
       </c>
       <c r="O24" s="18" t="n">
-        <v>57.17</v>
+        <v>-57.17</v>
       </c>
       <c r="P24" s="18" t="n">
         <v>-1.94</v>
@@ -2790,7 +2790,7 @@
         <v>3.43</v>
       </c>
       <c r="O25" s="18" t="n">
-        <v>45.49</v>
+        <v>-45.49</v>
       </c>
       <c r="P25" s="18" t="n">
         <v>-2.45</v>
@@ -2882,7 +2882,7 @@
         <v>5.4</v>
       </c>
       <c r="O26" s="18" t="n">
-        <v>42.69</v>
+        <v>-42.69</v>
       </c>
       <c r="P26" s="18" t="n">
         <v>-2.57</v>
@@ -2974,7 +2974,7 @@
         <v>4.53</v>
       </c>
       <c r="O27" s="18" t="n">
-        <v>64.56</v>
+        <v>-64.56</v>
       </c>
       <c r="P27" s="18" t="n">
         <v>-1.62</v>
@@ -3066,7 +3066,7 @@
         <v>5.17</v>
       </c>
       <c r="O28" s="18" t="n">
-        <v>62.18</v>
+        <v>-62.18</v>
       </c>
       <c r="P28" s="18" t="n">
         <v>-1.72</v>
@@ -3158,7 +3158,7 @@
         <v>5.4</v>
       </c>
       <c r="O29" s="18" t="n">
-        <v>65.28</v>
+        <v>-65.28</v>
       </c>
       <c r="P29" s="18" t="n">
         <v>-1.59</v>
@@ -3250,7 +3250,7 @@
         <v>5.94</v>
       </c>
       <c r="O30" s="18" t="n">
-        <v>71.04000000000001</v>
+        <v>-71.04000000000001</v>
       </c>
       <c r="P30" s="18" t="n">
         <v>-1.34</v>
@@ -3342,7 +3342,7 @@
         <v>6.24</v>
       </c>
       <c r="O31" s="18" t="n">
-        <v>55.05</v>
+        <v>-55.05</v>
       </c>
       <c r="P31" s="18" t="n">
         <v>-2.03</v>
@@ -3434,7 +3434,7 @@
         <v>4.73</v>
       </c>
       <c r="O32" s="18" t="n">
-        <v>49.29</v>
+        <v>-49.29</v>
       </c>
       <c r="P32" s="18" t="n">
         <v>-2.28</v>
@@ -3526,7 +3526,7 @@
         <v>9.34</v>
       </c>
       <c r="O33" s="18" t="n">
-        <v>40.2</v>
+        <v>-40.2</v>
       </c>
       <c r="P33" s="18" t="n">
         <v>-2.68</v>
@@ -3618,7 +3618,7 @@
         <v>2.17</v>
       </c>
       <c r="O34" s="18" t="n">
-        <v>53.76</v>
+        <v>-53.76</v>
       </c>
       <c r="P34" s="18" t="n">
         <v>-2.09</v>
@@ -3710,7 +3710,7 @@
         <v>3.15</v>
       </c>
       <c r="O35" s="18" t="n">
-        <v>51.25</v>
+        <v>-51.25</v>
       </c>
       <c r="P35" s="18" t="n">
         <v>-2.2</v>
@@ -3802,7 +3802,7 @@
         <v>10.13</v>
       </c>
       <c r="O36" s="18" t="n">
-        <v>44</v>
+        <v>-44</v>
       </c>
       <c r="P36" s="18" t="n">
         <v>-2.51</v>
@@ -3894,7 +3894,7 @@
         <v>9.19</v>
       </c>
       <c r="O37" s="18" t="n">
-        <v>46.63</v>
+        <v>-46.63</v>
       </c>
       <c r="P37" s="18" t="n">
         <v>-2.4</v>
@@ -3986,7 +3986,7 @@
         <v>4.57</v>
       </c>
       <c r="O38" s="18" t="n">
-        <v>44.85</v>
+        <v>-44.85</v>
       </c>
       <c r="P38" s="18" t="n">
         <v>-2.48</v>
@@ -4078,7 +4078,7 @@
         <v>6.1</v>
       </c>
       <c r="O39" s="18" t="n">
-        <v>44.68</v>
+        <v>-44.68</v>
       </c>
       <c r="P39" s="18" t="n">
         <v>-2.48</v>
@@ -4170,7 +4170,7 @@
         <v>4.54</v>
       </c>
       <c r="O40" s="18" t="n">
-        <v>41.61</v>
+        <v>-41.61</v>
       </c>
       <c r="P40" s="18" t="n">
         <v>-2.62</v>
@@ -4262,7 +4262,7 @@
         <v>6.66</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>49.9</v>
+        <v>-49.9</v>
       </c>
       <c r="P41" s="18" t="n">
         <v>-2.26</v>
@@ -4354,7 +4354,7 @@
         <v>6.49</v>
       </c>
       <c r="O42" s="18" t="n">
-        <v>45.72</v>
+        <v>-45.72</v>
       </c>
       <c r="P42" s="18" t="n">
         <v>-2.44</v>
@@ -4446,7 +4446,7 @@
         <v>6.48</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>39.49</v>
+        <v>-39.49</v>
       </c>
       <c r="P43" s="18" t="n">
         <v>-2.71</v>
@@ -4538,7 +4538,7 @@
         <v>5.56</v>
       </c>
       <c r="O44" s="18" t="n">
-        <v>61.43</v>
+        <v>-61.43</v>
       </c>
       <c r="P44" s="18" t="n">
         <v>-1.76</v>
@@ -4630,7 +4630,7 @@
         <v>5.56</v>
       </c>
       <c r="O45" s="18" t="n">
-        <v>57.07</v>
+        <v>-57.07</v>
       </c>
       <c r="P45" s="18" t="n">
         <v>-1.95</v>
@@ -4722,7 +4722,7 @@
         <v>10.25</v>
       </c>
       <c r="O46" s="18" t="n">
-        <v>60.11</v>
+        <v>-60.11</v>
       </c>
       <c r="P46" s="18" t="n">
         <v>-1.81</v>
@@ -4814,7 +4814,7 @@
         <v>4.19</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>46.38</v>
+        <v>-46.38</v>
       </c>
       <c r="P47" s="18" t="n">
         <v>-2.41</v>
@@ -4906,7 +4906,7 @@
         <v>16.3</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>51.66</v>
+        <v>-51.66</v>
       </c>
       <c r="P48" s="18" t="n">
         <v>-2.18</v>
@@ -4998,7 +4998,7 @@
         <v>4.69</v>
       </c>
       <c r="O49" s="18" t="n">
-        <v>58.25</v>
+        <v>-58.25</v>
       </c>
       <c r="P49" s="18" t="n">
         <v>-1.89</v>
@@ -5090,7 +5090,7 @@
         <v>2.48</v>
       </c>
       <c r="O50" s="18" t="n">
-        <v>51.91</v>
+        <v>-51.91</v>
       </c>
       <c r="P50" s="18" t="n">
         <v>-2.17</v>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Free energy released by Q -&gt; Q-.</t>
+          <t>Free energy of Q -&gt; Q-.</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>dG_Red / F - 4.42 V.</t>
+          <t>-dG_Red / F - 4.42 V.</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">

</xml_diff>